<commit_message>
Set container MSKU5698651 on the FOC declaration (JSD 3)
The FOC item ships inside MSKU5698651, not in a container of its own:
packing list 1 lists art. 0230238 (60 rolls, GW 2 720 kg) and its
footer reads MSKU5698651/CN6923658/20'GP/357PACKAGES/22470KGS/25CBM,
where the 357 packages include those 60 rolls.

JSD 3 now carries that container number in its label and container
column rather than as a parenthetical note, so the number goes on the
declaration. Notes restated: MSKU5698651 splits across JSD 1 and
JSD 3 (297 + 60 = 357 pcs, 19 750 + 2 720 = 22 470 kg), matching PL1
and the B/L; only MRKU9108387 is a clean one-container declaration.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EgFygQDzpiBueVLaTVai9C
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_ADITEG_CZ26009365.xlsx
+++ b/output/HS_Code_Summary_ADITEG_CZ26009365.xlsx
@@ -888,12 +888,12 @@
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>JSD 3 – FOC položka (kompenzace obj. 80615829)</t>
+          <t>JSD 3 – kontejner MSKU5698651 (FOC položka, kompenzace obj. 80615829)</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>MSKU5698651 (fyzicky v témže kontejneru jako JSD 1)</t>
+          <t>MSKU5698651</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
@@ -941,7 +941,7 @@
       <c r="A8" s="6" t="inlineStr"/>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>MEZISOUČET JSD 3 – FOC položka (kompenzace obj. 80615829)</t>
+          <t>MEZISOUČET JSD 3 – kontejner MSKU5698651 (FOC položka, kompenzace obj. 80615829)</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr"/>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>JSD 3 – FOC položka. POZOR: jede v kontejneru MSKU5698651 spolu s JSD 1, není to samostatný kontejner.</t>
+          <t>JSD 3 – FOC položka, kontejner MSKU5698651 (stejný kontejner jako JSD 1, dělí se mezi obě prohlášení).</t>
         </is>
       </c>
       <c r="G14" s="20" t="n"/>
@@ -2034,7 +2034,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A105"/>
+  <dimension ref="A1:A109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -2123,7 +2123,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>JSD 3 – FOC položka art. 0230238 (kompenzace obj. 80615829):</t>
+          <t>JSD 3 – kontejner MSKU5698651, FOC položka art. 0230238 (kompenzace obj. 80615829):</t>
         </is>
       </c>
     </row>
@@ -2147,475 +2147,475 @@
     <row r="17">
       <c r="A17" s="28" t="inlineStr">
         <is>
-          <t>⚠ POZOR – FOC ZBOŽÍ NENÍ SAMOSTATNÝ KONTEJNER</t>
+          <t>⚠ KONTEJNER U FOC POLOŽKY (JSD 3) = MSKU5698651</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Pravidlo „1 JSD = 1 kontejner“ platí pro JSD 1 a JSD 2. FOC položka (JSD 3) je fyzicky naložena</t>
+          <t>Na JSD 3 se do kolonky kontejneru uvádí MSKU5698651 – NE druhý kontejner a NE prázdná kolonka.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>v kontejneru MSKU5698651, tedy ve stejném kontejneru jako zboží na JSD 1.</t>
+          <t>Doklad: packing list 1 obsahuje FOC položku art. 0230238 (60 rolí, NW 2 700 kg, GW 2 720 kg)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Kontejner MSKU5698651 se proto dělí mezi dvě celní prohlášení:</t>
+          <t>a jeho patička uvádí: MSKU5698651/CN6923658/20'GP/357PACKAGES/22470KGS/25CBM.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">        JSD 1: 297 ks / GW 19 750 kg  +  JSD 3: 60 ks / GW 2 720 kg  =  357 ks / 22 470 kg</t>
+          <t>Celkem 357 kusů na PL1 zahrnuje i těchto 60 FOC rolí – FOC zboží tedy jede v tomto kontejneru.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="29" t="inlineStr">
-        <is>
-          <t>→ To přesně odpovídá packing listu 1 a údaji na B/L pro tento kontejner.</t>
-        </is>
-      </c>
+      <c r="A22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="29" t="inlineStr">
-        <is>
-          <t>→ Hmotnost kontejneru MSKU5698651 tedy NEBUDE souhlasit s JSD 1 samotným – je nutné uvádět</t>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Pravidlo „1 JSD = 1 kontejner“ proto platí beze zbytku jen pro JSD 2. Kontejner MSKU5698651</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">   obě JSD společně a v popisu zboží na obou uvést, že jde o dělený kontejner.</t>
+          <t>se dělí mezi dvě celní prohlášení (JSD 1 a JSD 3), obě na stejné číslo kontejneru:</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Kontejner MRKU9108387 = celé JSD 2, 172 ks / 22 420 kg – souhlasí bez dělení.</t>
+          <t xml:space="preserve">        JSD 1: 297 ks / GW 19 750 kg  +  JSD 3: 60 ks / GW 2 720 kg  =  357 ks / 22 470 kg</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
+      <c r="A26" s="29" t="inlineStr">
+        <is>
+          <t>→ To přesně odpovídá packing listu 1 i údaji na B/L pro tento kontejner.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="27" t="inlineStr">
-        <is>
-          <t>KONTROLA PROTI B/L AHD26060517</t>
+      <c r="A27" s="29" t="inlineStr">
+        <is>
+          <t>→ Hmotnost kontejneru NEBUDE souhlasit s JSD 1 samotným – v popisu zboží na JSD 1 i JSD 3</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t xml:space="preserve">   uvést, že jde o dělený kontejner, a obě prohlášení podat společně.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Kontejner MRKU9108387 = celé JSD 2, 172 ks / 22 420 kg – souhlasí bez dělení.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="27" t="inlineStr">
+        <is>
+          <t>KONTROLA PROTI B/L AHD26060517</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>B/L: 2 x 20'GP, 529 PACKAGES, 44 890,000 KGS, 50,000 CBM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="29" t="inlineStr">
-        <is>
-          <t>✓ Počet kusů: 297 + 172 + 60 = 529 ks – souhlasí.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="29" t="inlineStr">
-        <is>
-          <t>✓ Hrubá hmotnost: 19 750 + 22 420 + 2 720 = 44 890 kg – souhlasí na kilogram.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="29" t="inlineStr">
-        <is>
-          <t>✓ Kontejner MSKU5698651: 357 ks / 22 470 kg – souhlasí s B/L i PL1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="29" t="inlineStr">
-        <is>
-          <t>✓ Kontejner MRKU9108387: 172 ks / 22 420 kg – souhlasí s B/L i PL2.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="29" t="inlineStr">
         <is>
+          <t>✓ Počet kusů: 297 + 172 + 60 = 529 ks – souhlasí.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="29" t="inlineStr">
+        <is>
+          <t>✓ Hrubá hmotnost: 19 750 + 22 420 + 2 720 = 44 890 kg – souhlasí na kilogram.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="29" t="inlineStr">
+        <is>
+          <t>✓ Kontejner MSKU5698651: 357 ks / 22 470 kg – souhlasí s B/L i PL1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="29" t="inlineStr">
+        <is>
+          <t>✓ Kontejner MRKU9108387: 172 ks / 22 420 kg – souhlasí s B/L i PL2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="29" t="inlineStr">
+        <is>
           <t>✓ Součty faktur: 10 503,01 + 13 651,81 = 24 154,82 USD (bez FOC).</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="27" t="inlineStr">
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="27" t="inlineStr">
         <is>
           <t>CELNÍ HODNOTA – pravidlo „Total“</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+    <row r="40">
+      <c r="A40" t="inlineStr">
         <is>
           <t>Použity částky ze sloupce „Total amount usd“ na fakturách. Žádná obchodní sleva na této zásilce není,</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>hodnoty před/po slevě se tedy neuvádějí. Kontrolní součty JSD 1 a JSD 2 odpovídají řádku „Total“ faktur.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>FOC položka nemá na faktuře hodnotu (0,00) – celní hodnota dopočtena, viz JSD 3.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="30" t="inlineStr">
-        <is>
-          <t>⚠ SAZEBNÍ ZAŘAZENÍ – POUŽITO PRAVIDLO CCT/VPV KN</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>V podkladech (faktury, packing listy, B/L) NENÍ uveden žádný HS kód – B/L popisuje zboží jen jako</t>
+          <t>hodnoty před/po slevě se tedy neuvádějí. Kontrolní součty JSD 1 a JSD 2 odpovídají řádku „Total“ faktur.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>„RUBBER SHEET“. Oba níže uvedené kódy jsem odvodila pravidlem CCT/VPV KN podle</t>
+          <t>FOC položka nemá na faktuře hodnotu (0,00) – celní hodnota dopočtena, viz JSD 3.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>reference/Common_Customs_Tariff_EU_CZ.pptx. Takto zařazené položky:</t>
-        </is>
-      </c>
+      <c r="A43" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr"/>
+      <c r="A44" s="30" t="inlineStr">
+        <is>
+          <t>⚠ SAZEBNÍ ZAŘAZENÍ – POUŽITO PRAVIDLO CCT/VPV KN</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>A) 4008 21 90 – art. 0231268, 0230179, 0231419, 0230264, 0234614, 0230540, 0232061,</t>
+          <t>V podkladech (faktury, packing listy, B/L) NENÍ uveden žádný HS kód – B/L popisuje zboží jen jako</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">   0232184, 0231843, 0231842, 0230301</t>
+          <t>„RUBBER SHEET“. Oba níže uvedené kódy jsem odvodila pravidlem CCT/VPV KN podle</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">   CO TO JE? Desky / pásy z vulkanizovaného kaučuku v rolích, černé, 65 ±5 ShA, 2-3 a 7-8 MPa, tl. 3–20 mm.</t>
+          <t>reference/Common_Customs_Tariff_EU_CZ.pptx. Takto zařazené položky:</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Z ČEHO TO JE? Vulkanizovaný nelehčený kaučuk SBR / EPDM; u tří položek 1 textilní vložka (fabric) jako výztuž.</t>
-        </is>
-      </c>
+      <c r="A48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">   K ČEMU SLOUŽÍ? Technická pryž – těsnění, obklady, podložky; polotovar dodávaný v rolích k dalšímu zpracování.</t>
+          <t>A) 4008 21 90 – art. 0231268, 0230179, 0231419, 0230264, 0234614, 0230540, 0232061,</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Postup: TŘÍDA VII (plasty, kaučuk a pryž) → kapitola 40 → úvodní poznámky ke kap. 40 zboží nevylučují →</t>
+          <t xml:space="preserve">   0232184, 0231843, 0231842, 0230301</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">   číslo 4008 „Desky, listy, pásy, tyče a profily z vulkanizovaného kaučuku, jiného než tvrdého kaučuku“ →</t>
+          <t xml:space="preserve">   CO TO JE? Desky / pásy z vulkanizovaného kaučuku v rolích, černé, 65 ±5 ShA, 2-3 a 7-8 MPa, tl. 3–20 mm.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">   podpoložka 4008 21 (z nelehčeného kaučuku – desky, listy a pásy) → KN 4008 21 90 (ostatní). VPV 1 a VPV 6.</t>
+          <t xml:space="preserve">   Z ČEHO TO JE? Vulkanizovaný nelehčený kaučuk SBR / EPDM; u tří položek 1 textilní vložka (fabric) jako výztuž.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Textilní vložka: podle VPV 3(b) dává podstatný charakter kaučuk (výrazně převažuje hmotnostně, vložka</t>
+          <t xml:space="preserve">   K ČEMU SLOUŽÍ? Technická pryž – těsnění, obklady, podložky; polotovar dodávaný v rolích k dalšímu zpracování.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">   plní pouze vyztužovací funkci) → zůstává v kap. 40, nikoli v kap. 59.</t>
+          <t xml:space="preserve">   Postup: TŘÍDA VII (plasty, kaučuk a pryž) → kapitola 40 → úvodní poznámky ke kap. 40 zboží nevylučují →</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr"/>
+      <c r="A55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   číslo 4008 „Desky, listy, pásy, tyče a profily z vulkanizovaného kaučuku, jiného než tvrdého kaučuku“ →</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>B) 4016 91 00 – art. 0230559, 0230564, 0230238</t>
+          <t xml:space="preserve">   podpoložka 4008 21 (z nelehčeného kaučuku – desky, listy a pásy) → KN 4008 21 90 (ostatní). VPV 1 a VPV 6.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">   CO TO JE? Podlahové rohože z pryže – kamínková deska, kamínková deska speciál, rýhovaná deska.</t>
+          <t xml:space="preserve">   Textilní vložka: podle VPV 3(b) dává podstatný charakter kaučuk (výrazně převažuje hmotnostně, vložka</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Z ČEHO TO JE? Vulkanizovaný nelehčený kaučuk (pryž).</t>
+          <t xml:space="preserve">   plní pouze vyztužovací funkci) → zůstává v kap. 40, nikoli v kap. 59.</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   K ČEMU SLOUŽÍ? Podlahová krytina / rohož – stájové a protiskluzové podlahy (Horse Rubber mat, Stable Mat).</t>
-        </is>
-      </c>
+      <c r="A59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Postup: TŘÍDA VII → kapitola 40 → číslo 4016 „Ostatní výrobky z vulkanizovaného kaučuku, jiného než</t>
+          <t>B) 4016 91 00 – art. 0230559, 0230564, 0230238</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">   tvrdého kaučuku“ → KN 4016 91 00 „Podlahové krytiny a rohože“. Podle VPV 3(a) má konkrétnější popis</t>
+          <t xml:space="preserve">   CO TO JE? Podlahové rohože z pryže – kamínková deska, kamínková deska speciál, rýhovaná deska.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">   (hotová podlahová krytina) přednost před obecným číslem 4008 pro desky a pásy.</t>
+          <t xml:space="preserve">   Z ČEHO TO JE? Vulkanizovaný nelehčený kaučuk (pryž).</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr"/>
+      <c r="A63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   K ČEMU SLOUŽÍ? Podlahová krytina / rohož – stájové a protiskluzové podlahy (Horse Rubber mat, Stable Mat).</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" s="30" t="inlineStr">
-        <is>
-          <t>⚠ NEJISTOTA – DOPORUČUJI KONZULTOVAT</t>
+      <c r="A64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Postup: TŘÍDA VII → kapitola 40 → číslo 4016 „Ostatní výrobky z vulkanizovaného kaučuku, jiného než</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>1) Hranice 4008 vs. 4016 u art. 0230559 (3 mm Kamínková deska, dodávaná v roli 1,2 × 10 m) – rozměr</t>
+          <t xml:space="preserve">   tvrdého kaučuku“ → KN 4016 91 00 „Podlahové krytiny a rohože“. Podle VPV 3(a) má konkrétnější popis</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">   odpovídá spíše roli materiálu než hotové rohoži. Zařazeno do 4016 91 00 podle účelu (stájová rohož).</t>
+          <t xml:space="preserve">   (hotová podlahová krytina) přednost před obecným číslem 4008 pro desky a pásy.</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>2) Položky s textilní vložkou – hranice kap. 40 vs. 5906. Zařazeno do 4008 21 90.</t>
-        </is>
-      </c>
+      <c r="A67" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="29" t="inlineStr">
-        <is>
-          <t>→ Před podáním doporučuji potvrdit v TARIC, případně konzultovat tarifní tým: customs.tariff@mauriceward.com</t>
+      <c r="A68" s="30" t="inlineStr">
+        <is>
+          <t>⚠ NEJISTOTA – DOPORUČUJI KONZULTOVAT</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">   (tento krok jsem zatím neprovedla – rozhodni prosím Ty).</t>
+          <t>1) Hranice 4008 vs. 4016 u art. 0230559 (3 mm Kamínková deska, dodávaná v roli 1,2 × 10 m) – rozměr</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr"/>
+      <c r="A70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   odpovídá spíše roli materiálu než hotové rohoži. Zařazeno do 4016 91 00 podle účelu (stájová rohož).</t>
+        </is>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="28" t="inlineStr">
-        <is>
-          <t>⚠ PREFERENČNÍ PŮVOD A REX – OBOJÍ CHYBÍ</t>
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2) Položky s textilní vložkou – hranice kap. 40 vs. 5906. Zařazeno do 4008 21 90.</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>PREFERENČNÍ VĚTA: NENÍ uvedena v žádném z dokladů. Zkontrolovány obě faktury, oba packing listy i B/L.</t>
+      <c r="A72" s="29" t="inlineStr">
+        <is>
+          <t>→ Před podáním doporučuji potvrdit v TARIC, případně konzultovat tarifní tým: customs.tariff@mauriceward.com</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>REX ČÍSLO: NENÍ na žádné z faktur uvedeno. Faktury neobsahují číslo registrovaného vývozce</t>
+          <t xml:space="preserve">   (tento krok jsem zatím neprovedla – rozhodni prosím Ty).</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>ani jiné číslo celního povolení vývozce.</t>
-        </is>
-      </c>
+      <c r="A74" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Země původu: Čína (CN). EU nemá s ČLR dohodu o preferenčním obchodu, preferenční sazba proto</t>
+      <c r="A75" s="28" t="inlineStr">
+        <is>
+          <t>⚠ PREFERENČNÍ PŮVOD A REX – OBOJÍ CHYBÍ</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>není možná ani při doložení prohlášení – uplatní se standardní třetizemní clo (erga omnes).</t>
+          <t>PREFERENČNÍ VĚTA: NENÍ uvedena v žádném z dokladů. Zkontrolovány obě faktury, oba packing listy i B/L.</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="29" t="inlineStr">
-        <is>
-          <t>→ Sazbu k oběma HS kódům ověřit v TARIC k datu propuštění zboží.</t>
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>REX ČÍSLO: NENÍ na žádné z faktur uvedeno. Faktury neobsahují číslo registrovaného vývozce</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr"/>
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>ani jiné číslo celního povolení vývozce.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
-      <c r="A79" s="30" t="inlineStr">
-        <is>
-          <t>CBAM</t>
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Země původu: Čína (CN). EU nemá s ČLR dohodu o preferenčním obchodu, preferenční sazba proto</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
+          <t>není možná ani při doložení prohlášení – uplatní se standardní třetizemní clo (erga omnes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="29" t="inlineStr">
+        <is>
+          <t>→ Sazbu k oběma HS kódům ověřit v TARIC k datu propuštění zboží.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="30" t="inlineStr">
+        <is>
+          <t>CBAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
           <t>Zásilka NEOBSAHUJE žádnou CBAM položku – kaučuk a pryž (kapitola 40) nejsou v příloze I nařízení CBAM</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>(CBAM = cement, elektřina, hnojiva, železo a ocel, hliník, vodík). Kód Y128/Y238/Y137 se na žádné JSD neuvádí.</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>Pro pořádek prověřeno v reference/CBAM_receivers_CZ.xlsx (list List1):</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="31" t="inlineStr">
-        <is>
-          <t>⚠ ADITEG s.r.o. (EORI CZ26905710) V REGISTRU NENÍ – ani podle názvu firmy, ani podle EORI.</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="29" t="inlineStr">
-        <is>
-          <t>→ Pro tuto zásilku to nevadí (žádné CBAM zboží). Pokud by ADITEG někdy dovážel CBAM zboží, je nutné</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">   nejdřív zjistit jeho CBAM status a doplnit ho do registru. Status nedomýšlet.</t>
+          <t>(CBAM = cement, elektřina, hnojiva, železo a ocel, hliník, vodík). Kód Y128/Y238/Y137 se na žádné JSD neuvádí.</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr"/>
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Pro pořádek prověřeno v reference/CBAM_receivers_CZ.xlsx (list List1):</t>
+        </is>
+      </c>
     </row>
     <row r="87">
-      <c r="A87" s="30" t="inlineStr">
-        <is>
-          <t>ANTIDUMPING</t>
+      <c r="A87" s="31" t="inlineStr">
+        <is>
+          <t>⚠ ADITEG s.r.o. (EORI CZ26905710) V REGISTRU NENÍ – ani podle názvu firmy, ani podle EORI.</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>Pro desky a rohože z vulkanizovaného kaučuku (4008 21, 4016 91) původem z ČLR nebylo zjištěno</t>
+      <c r="A88" s="29" t="inlineStr">
+        <is>
+          <t>→ Pro tuto zásilku to nevadí (žádné CBAM zboží). Pokud by ADITEG někdy dovážel CBAM zboží, je nutné</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>žádné platné antidumpingové ani vyrovnávací opatření. Ověřit v TARIC k datu podání JSD.</t>
+          <t xml:space="preserve">   nejdřív zjistit jeho CBAM status a doplnit ho do registru. Status nedomýšlet.</t>
         </is>
       </c>
     </row>
@@ -2625,21 +2625,21 @@
     <row r="91">
       <c r="A91" s="30" t="inlineStr">
         <is>
-          <t>INCOTERM</t>
+          <t>ANTIDUMPING</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>FOB Xingang (Tianjin), Čína – dle obou faktur. Na B/L „FREIGHT COLLECT“, což je s FOB v souladu.</t>
+          <t>Pro desky a rohože z vulkanizovaného kaučuku (4008 21, 4016 91) původem z ČLR nebylo zjištěno</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="29" t="inlineStr">
-        <is>
-          <t>→ Do celní hodnoty je nutno připočíst náklady na přepravu a pojištění do místa vstupu do EU.</t>
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>žádné platné antidumpingové ani vyrovnávací opatření. Ověřit v TARIC k datu podání JSD.</t>
         </is>
       </c>
     </row>
@@ -2647,73 +2647,97 @@
       <c r="A94" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" s="28" t="inlineStr">
-        <is>
-          <t>⚠ NESROVNALOST V PODKLADECH – art. 0230564</t>
+      <c r="A95" s="30" t="inlineStr">
+        <is>
+          <t>INCOTERM</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
+          <t>FOB Xingang (Tianjin), Čína – dle obou faktur. Na B/L „FREIGHT COLLECT“, což je s FOB v souladu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="29" t="inlineStr">
+        <is>
+          <t>→ Do celní hodnoty je nutno připočíst náklady na přepravu a pojištění do místa vstupu do EU.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="28" t="inlineStr">
+        <is>
+          <t>⚠ NESROVNALOST V PODKLADECH – art. 0230564</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
           <t>Faktura uvádí „17 mm Kamínková deska spec.“, packing list v popisu „12 mm Kamínková deska spec.“,</t>
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
+    <row r="101">
+      <c r="A101" t="inlineStr">
         <is>
           <t>přičemž rozměr je v obou dokladech 1,22 x 1,83 m x 17 mm. V tabulce je použit popis z faktury (17 mm).</t>
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="29" t="inlineStr">
+    <row r="102">
+      <c r="A102" s="29" t="inlineStr">
         <is>
           <t>→ Vyjasnit s odesílatelem před podáním – údaj jde do popisu zboží v kolonce 31.</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
-        <is>
-          <t>Kontrola množství: 446,52 m² / (1,22 × 1,83 m) = přesně 200 ks – souhlasí s packing listem.</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr"/>
-    </row>
-    <row r="101">
-      <c r="A101" s="27" t="inlineStr">
-        <is>
-          <t>POZNÁMKA K POPISU ZBOŽÍ A KE SLUČOVÁNÍ</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>Popisy v tabulce jsou převzaty doslovně z faktur (česky), bez úprav a bez přeformulování.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
+          <t>Kontrola množství: 446,52 m² / (1,22 × 1,83 m) = přesně 200 ks – souhlasí s packing listem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="27" t="inlineStr">
+        <is>
+          <t>POZNÁMKA K POPISU ZBOŽÍ A KE SLUČOVÁNÍ</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Popisy v tabulce jsou převzaty doslovně z faktur (česky), bez úprav a bez přeformulování.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
           <t>Položky jsou sloučeny na unikátní HS kódy v rámci každého JSD. Stejný HS kód 4008 21 90 je na JSD 1</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
+    <row r="108">
+      <c r="A108" t="inlineStr">
         <is>
           <t>i na JSD 2 samostatně – jde o dvě různá celní prohlášení, nelze je slučovat napříč JSD.</t>
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
+    <row r="109">
+      <c r="A109" t="inlineStr">
         <is>
           <t>Odesílatel je u celé zásilky jeden (Qingdao Conet), dělení podle odesílatele proto nebylo potřeba.</t>
         </is>

</xml_diff>

<commit_message>
Use a single HS code 4008 21 90 for the whole shipment
Per the declarant, all 15 invoice lines across the three declarations
go under 4008 21 90. This merges the items previously classified as
4016 91 00 (art. 0230559, 0230564 and the FOC art. 0230238) into the
same code, leaving one HS row per JSD.

The notes now record the code as supplied by the declarant rather
than derived, while keeping the fact that no HS code appears in any
of the sender's documents and a short record that 4016 91 00 was the
considered alternative for the mats. Antidumping note narrowed to the
code actually declared.

Quantities, weights and values are unchanged and still reconcile with
the B/L (529 pcs / 44 890 kg) and the invoice Total lines.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EgFygQDzpiBueVLaTVai9C
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_ADITEG_CZ26009365.xlsx
+++ b/output/HS_Code_Summary_ADITEG_CZ26009365.xlsx
@@ -555,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:M18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -667,7 +667,9 @@
 0230179 – SBR 65 +/- 5 Sh.černá, 2-3 MPa 5 mm x 1.200 x 10.000 mm
 0231419 – SBR 65 +/- 5 Sh.černá, 2-3 MPa 6 mm x 2.000 x 10.000 mm
 0230264 – SBR 65 +/- 5 Sh.černá, 2-3 MPa, 1 vložka(fabric) 10 mm x 1.200 x 10.000 mm
-0234614 – SBR 65 +/-5SHA  černá, 2-3 MPa 8 mm x1.600 x 10.000 mm</t>
+0234614 – SBR 65 +/-5SHA  černá, 2-3 MPa 8 mm x1.600 x 10.000 mm
+0230559 – 3 mm Kamínková deska.(Horse Rubber mat) 3 mm x 1.200 x 10.000 mm
+0230564 – 17 mm Kamínková deska spec.（Round button Stable Mat）Kamínková deska - speciál 1,22 x 1,83 m x 17 mm</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -676,19 +678,19 @@
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1268</v>
+        <v>1786.52</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>91</v>
+        <v>297</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>11018</v>
+        <v>19379</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>11220</v>
+        <v>19750</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>5374.71</v>
+        <v>10503.01</v>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
@@ -697,119 +699,61 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>HS kód odvozen pravidlem CCT/VPV KN (v podkladech není uveden) – ověřit v TARIC. U položek s textilní vložkou (0230264, 0232184, 0230301) ověřit hranici vůči kap. 59 (5906).</t>
+          <t>HS kód zadán deklarantem – celá zásilka pod jedním kódem 4008 21 90. V podkladech odesílatele HS kód uveden není.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr"/>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>MEZISOUČET JSD 1 – kontejner MSKU5698651 (placené zboží)</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr"/>
+      <c r="D3" s="6" t="inlineStr"/>
+      <c r="E3" s="6" t="inlineStr"/>
+      <c r="F3" s="6" t="inlineStr"/>
+      <c r="G3" s="7" t="n">
+        <v>1786.52</v>
+      </c>
+      <c r="H3" s="8" t="n">
+        <v>297</v>
+      </c>
+      <c r="I3" s="7" t="n">
+        <v>19379</v>
+      </c>
+      <c r="J3" s="7" t="n">
+        <v>19750</v>
+      </c>
+      <c r="K3" s="7" t="n">
+        <v>10503.01</v>
+      </c>
+      <c r="L3" s="6" t="inlineStr"/>
+      <c r="M3" s="6" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>Qingdao Conet International Trade Co., Ltd., Qingdao, ČLR</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>JSD 1 – kontejner MSKU5698651 (placené zboží)</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>MSKU5698651</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>4016910000</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>0230559 – 3 mm Kamínková deska.(Horse Rubber mat) 3 mm x 1.200 x 10.000 mm
-0230564 – 17 mm Kamínková deska spec.（Round button Stable Mat）Kamínková deska - speciál 1,22 x 1,83 m x 17 mm</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>518.52</v>
-      </c>
-      <c r="H3" s="5" t="n">
-        <v>206</v>
-      </c>
-      <c r="I3" s="4" t="n">
-        <v>8361</v>
-      </c>
-      <c r="J3" s="4" t="n">
-        <v>8530</v>
-      </c>
-      <c r="K3" s="4" t="n">
-        <v>5128.3</v>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>FOB Xingang (Tianjin), Čína</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>HS kód odvozen pravidlem CCT/VPV KN (v podkladech není uveden) – ověřit v TARIC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr"/>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>MEZISOUČET JSD 1 – kontejner MSKU5698651 (placené zboží)</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="7" t="n">
-        <v>1786.52</v>
-      </c>
-      <c r="H4" s="8" t="n">
-        <v>297</v>
-      </c>
-      <c r="I4" s="7" t="n">
-        <v>19379</v>
-      </c>
-      <c r="J4" s="7" t="n">
-        <v>19750</v>
-      </c>
-      <c r="K4" s="7" t="n">
-        <v>10503.01</v>
-      </c>
-      <c r="L4" s="6" t="inlineStr"/>
-      <c r="M4" s="6" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Qingdao Conet International Trade Co., Ltd., Qingdao, ČLR</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>JSD 2 – kontejner MRKU9108387 (placené zboží)</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>MRKU9108387</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>4008219000</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>0230540 – EPDM/SBR 65 +/- 5 Sh.černá, 7-8 MPa 5mm x 1.200 x 10.000 mm
 0232061 – SBR 65 +/- 5 Sh. černá, 2-3 MPa 20 mm x 1.400 x 10.000 mm
@@ -820,186 +764,199 @@
 0230301 – EPDM/SBR 65 +/- 5 ShA černá, 2-3 MPa, 1 vložka 8 mm x 1.200 x 10.000 mm</t>
         </is>
       </c>
-      <c r="F5" s="10" t="inlineStr">
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="G5" s="11" t="n">
+      <c r="G4" s="11" t="n">
         <v>2392</v>
       </c>
-      <c r="H5" s="12" t="n">
+      <c r="H4" s="12" t="n">
         <v>172</v>
       </c>
-      <c r="I5" s="11" t="n">
+      <c r="I4" s="11" t="n">
         <v>22340</v>
       </c>
-      <c r="J5" s="11" t="n">
+      <c r="J4" s="11" t="n">
         <v>22420</v>
       </c>
-      <c r="K5" s="11" t="n">
+      <c r="K4" s="11" t="n">
         <v>13651.81</v>
       </c>
-      <c r="L5" s="9" t="inlineStr">
+      <c r="L4" s="9" t="inlineStr">
         <is>
           <t>FOB Xingang (Tianjin), Čína</t>
         </is>
       </c>
-      <c r="M5" s="9" t="inlineStr">
-        <is>
-          <t>HS kód odvozen pravidlem CCT/VPV KN (v podkladech není uveden) – ověřit v TARIC. U položek s textilní vložkou (0230264, 0232184, 0230301) ověřit hranici vůči kap. 59 (5906).</t>
-        </is>
-      </c>
+      <c r="M4" s="9" t="inlineStr">
+        <is>
+          <t>HS kód zadán deklarantem – celá zásilka pod jedním kódem 4008 21 90. V podkladech odesílatele HS kód uveden není.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr"/>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>MEZISOUČET JSD 2 – kontejner MRKU9108387 (placené zboží)</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr"/>
+      <c r="D5" s="6" t="inlineStr"/>
+      <c r="E5" s="6" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr"/>
+      <c r="G5" s="7" t="n">
+        <v>2392</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>172</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>22340</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>22420</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>13651.81</v>
+      </c>
+      <c r="L5" s="6" t="inlineStr"/>
+      <c r="M5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr"/>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>MEZISOUČET JSD 2 – kontejner MRKU9108387 (placené zboží)</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="7" t="n">
-        <v>2392</v>
-      </c>
-      <c r="H6" s="8" t="n">
-        <v>172</v>
-      </c>
-      <c r="I6" s="7" t="n">
-        <v>22340</v>
-      </c>
-      <c r="J6" s="7" t="n">
-        <v>22420</v>
-      </c>
-      <c r="K6" s="7" t="n">
-        <v>13651.81</v>
-      </c>
-      <c r="L6" s="6" t="inlineStr"/>
-      <c r="M6" s="6" t="inlineStr"/>
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Qingdao Conet International Trade Co., Ltd., Qingdao, ČLR</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>JSD 3 – kontejner MSKU5698651 (FOC položka, kompenzace obj. 80615829)</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>MSKU5698651</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>4008219000</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>0230238 – Fine ribbed mat(Rýhovaná deska - malá) 3mm，1.2X10m</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>CN</t>
+        </is>
+      </c>
+      <c r="G6" s="15" t="n">
+        <v>720</v>
+      </c>
+      <c r="H6" s="16" t="n">
+        <v>60</v>
+      </c>
+      <c r="I6" s="15" t="n">
+        <v>2700</v>
+      </c>
+      <c r="J6" s="15" t="n">
+        <v>2720</v>
+      </c>
+      <c r="K6" s="15" t="n">
+        <v>1928.45</v>
+      </c>
+      <c r="L6" s="13" t="inlineStr">
+        <is>
+          <t>FOB Xingang (Tianjin), Čína</t>
+        </is>
+      </c>
+      <c r="M6" s="13" t="inlineStr">
+        <is>
+          <t>FOC – na faktuře 0,00 USD. Celní hodnota dopočtena z jednotkové ceny stejného zboží na faktuře: 2,6784 USD/m² × 720 m² = 1 928,448 USD. Odsouhlaseno. HS kód zadán deklarantem – celá zásilka pod jedním kódem 4008 21 90. V podkladech odesílatele HS kód uveden není.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t>Qingdao Conet International Trade Co., Ltd., Qingdao, ČLR</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>JSD 3 – kontejner MSKU5698651 (FOC položka, kompenzace obj. 80615829)</t>
-        </is>
-      </c>
-      <c r="C7" s="13" t="inlineStr">
-        <is>
-          <t>MSKU5698651</t>
-        </is>
-      </c>
-      <c r="D7" s="14" t="inlineStr">
-        <is>
-          <t>4016910000</t>
-        </is>
-      </c>
-      <c r="E7" s="13" t="inlineStr">
-        <is>
-          <t>0230238 – Fine ribbed mat(Rýhovaná deska - malá) 3mm，1.2X10m</t>
-        </is>
-      </c>
-      <c r="F7" s="14" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="G7" s="15" t="n">
+      <c r="A7" s="6" t="inlineStr"/>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>MEZISOUČET JSD 3 – kontejner MSKU5698651 (FOC položka, kompenzace obj. 80615829)</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr"/>
+      <c r="D7" s="6" t="inlineStr"/>
+      <c r="E7" s="6" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="7" t="n">
         <v>720</v>
       </c>
-      <c r="H7" s="16" t="n">
+      <c r="H7" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="I7" s="15" t="n">
+      <c r="I7" s="7" t="n">
         <v>2700</v>
       </c>
-      <c r="J7" s="15" t="n">
+      <c r="J7" s="7" t="n">
         <v>2720</v>
       </c>
-      <c r="K7" s="15" t="n">
+      <c r="K7" s="7" t="n">
         <v>1928.45</v>
       </c>
-      <c r="L7" s="13" t="inlineStr">
-        <is>
-          <t>FOB Xingang (Tianjin), Čína</t>
-        </is>
-      </c>
-      <c r="M7" s="13" t="inlineStr">
-        <is>
-          <t>FOC – na faktuře 0,00 USD. Celní hodnota dopočtena z jednotkové ceny stejného zboží na faktuře: 2,6784 USD/m² × 720 m² = 1 928,448 USD. Odsouhlaseno. HS kód odvozen pravidlem CCT/VPV KN (v podkladech není uveden) – ověřit v TARIC.</t>
-        </is>
-      </c>
+      <c r="L7" s="6" t="inlineStr"/>
+      <c r="M7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr"/>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>MEZISOUČET JSD 3 – kontejner MSKU5698651 (FOC položka, kompenzace obj. 80615829)</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr"/>
-      <c r="D8" s="6" t="inlineStr"/>
-      <c r="E8" s="6" t="inlineStr"/>
-      <c r="F8" s="6" t="inlineStr"/>
-      <c r="G8" s="7" t="n">
-        <v>720</v>
-      </c>
-      <c r="H8" s="8" t="n">
-        <v>60</v>
-      </c>
-      <c r="I8" s="7" t="n">
-        <v>2700</v>
-      </c>
-      <c r="J8" s="7" t="n">
-        <v>2720</v>
-      </c>
-      <c r="K8" s="7" t="n">
-        <v>1928.45</v>
-      </c>
-      <c r="L8" s="6" t="inlineStr"/>
-      <c r="M8" s="6" t="inlineStr"/>
+      <c r="A8" s="17" t="inlineStr"/>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>CELKEM ZÁSILKA</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr"/>
+      <c r="D8" s="17" t="inlineStr"/>
+      <c r="E8" s="17" t="inlineStr"/>
+      <c r="F8" s="17" t="inlineStr"/>
+      <c r="G8" s="18" t="n">
+        <v>4898.52</v>
+      </c>
+      <c r="H8" s="19" t="n">
+        <v>529</v>
+      </c>
+      <c r="I8" s="18" t="n">
+        <v>44419</v>
+      </c>
+      <c r="J8" s="18" t="n">
+        <v>44890</v>
+      </c>
+      <c r="K8" s="18" t="n">
+        <v>26083.27</v>
+      </c>
+      <c r="L8" s="17" t="inlineStr"/>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>Souhlasí s B/L AHD26060517: 529 PACKAGES / 44 890,000 KGS</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr"/>
-      <c r="B9" s="17" t="inlineStr">
-        <is>
-          <t>CELKEM ZÁSILKA</t>
-        </is>
-      </c>
-      <c r="C9" s="17" t="inlineStr"/>
-      <c r="D9" s="17" t="inlineStr"/>
-      <c r="E9" s="17" t="inlineStr"/>
-      <c r="F9" s="17" t="inlineStr"/>
-      <c r="G9" s="18" t="n">
-        <v>4898.52</v>
-      </c>
-      <c r="H9" s="19" t="n">
-        <v>529</v>
-      </c>
-      <c r="I9" s="18" t="n">
-        <v>44419</v>
-      </c>
-      <c r="J9" s="18" t="n">
-        <v>44890</v>
-      </c>
-      <c r="K9" s="18" t="n">
-        <v>26083.27</v>
-      </c>
-      <c r="L9" s="17" t="inlineStr"/>
-      <c r="M9" s="17" t="inlineStr">
-        <is>
-          <t>Souhlasí s B/L AHD26060517: 529 PACKAGES / 44 890,000 KGS</t>
-        </is>
-      </c>
+      <c r="G9" s="20" t="n"/>
+      <c r="H9" s="21" t="n"/>
+      <c r="I9" s="20" t="n"/>
+      <c r="J9" s="20" t="n"/>
+      <c r="K9" s="20" t="n"/>
     </row>
     <row r="10">
+      <c r="A10" s="22" t="inlineStr">
+        <is>
+          <t>Legenda:</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
       <c r="G10" s="20" t="n"/>
       <c r="H10" s="21" t="n"/>
       <c r="I10" s="20" t="n"/>
@@ -1009,10 +966,14 @@
     <row r="11">
       <c r="A11" s="22" t="inlineStr">
         <is>
-          <t>Legenda:</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
+          <t>🔵 MODRÁ</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>JSD 1 – kontejner MSKU5698651, placené zboží.</t>
+        </is>
+      </c>
       <c r="G11" s="20" t="n"/>
       <c r="H11" s="21" t="n"/>
       <c r="I11" s="20" t="n"/>
@@ -1022,12 +983,12 @@
     <row r="12">
       <c r="A12" s="22" t="inlineStr">
         <is>
-          <t>🔵 MODRÁ</t>
+          <t>🟢 ZELENÁ</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>JSD 1 – kontejner MSKU5698651, placené zboží.</t>
+          <t>JSD 2 – kontejner MRKU9108387, placené zboží.</t>
         </is>
       </c>
       <c r="G12" s="20" t="n"/>
@@ -1039,12 +1000,12 @@
     <row r="13">
       <c r="A13" s="22" t="inlineStr">
         <is>
-          <t>🟢 ZELENÁ</t>
+          <t>🟠 ORANŽOVÁ</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>JSD 2 – kontejner MRKU9108387, placené zboží.</t>
+          <t>JSD 3 – FOC položka, kontejner MSKU5698651 (stejný kontejner jako JSD 1, dělí se mezi obě prohlášení).</t>
         </is>
       </c>
       <c r="G13" s="20" t="n"/>
@@ -1056,12 +1017,12 @@
     <row r="14">
       <c r="A14" s="22" t="inlineStr">
         <is>
-          <t>🟠 ORANŽOVÁ</t>
+          <t>HS kód</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>JSD 3 – FOC položka, kontejner MSKU5698651 (stejný kontejner jako JSD 1, dělí se mezi obě prohlášení).</t>
+          <t>Celá zásilka pod jedním kódem 4008 21 90 – zadáno deklarantem. V podkladech odesílatele HS kód není.</t>
         </is>
       </c>
       <c r="G14" s="20" t="n"/>
@@ -1073,12 +1034,12 @@
     <row r="15">
       <c r="A15" s="22" t="inlineStr">
         <is>
-          <t>⚠ HS kódy</t>
+          <t>⚠ Preferenční věta</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>V podkladech NEJSOU uvedeny – odvozeny pravidlem CCT/VPV KN. Viz list „Dokumenty a poznámky“.</t>
+          <t>V dokladech NENÍ. ⚠ REX číslo na fakturách také NENÍ. Původ ČLR → standardní třetizemní clo.</t>
         </is>
       </c>
       <c r="G15" s="20" t="n"/>
@@ -1090,12 +1051,12 @@
     <row r="16">
       <c r="A16" s="22" t="inlineStr">
         <is>
-          <t>⚠ Preferenční věta</t>
+          <t>Celní hodnota</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>V dokladech NENÍ. ⚠ REX číslo na fakturách také NENÍ. Původ ČLR → standardní třetizemní clo.</t>
+          <t>Převzata ze sloupce „Total amount usd“ na fakturách. Žádná sleva se neuplatňuje.</t>
         </is>
       </c>
       <c r="G16" s="20" t="n"/>
@@ -1107,12 +1068,12 @@
     <row r="17">
       <c r="A17" s="22" t="inlineStr">
         <is>
-          <t>Celní hodnota</t>
+          <t>Popis zboží</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Převzata ze sloupce „Total amount usd“ na fakturách. Žádná sleva se neuplatňuje.</t>
+          <t>Doslovný český popis z faktury, bez úprav.</t>
         </is>
       </c>
       <c r="G17" s="20" t="n"/>
@@ -1124,12 +1085,12 @@
     <row r="18">
       <c r="A18" s="22" t="inlineStr">
         <is>
-          <t>Popis zboží</t>
+          <t>CBAM</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Doslovný český popis z faktury, bez úprav.</t>
+          <t>Netýká se (kapitola 40). ⚠ ADITEG s.r.o. však v registru CBAM chybí – viz poznámky.</t>
         </is>
       </c>
       <c r="G18" s="20" t="n"/>
@@ -1137,23 +1098,6 @@
       <c r="I18" s="20" t="n"/>
       <c r="J18" s="20" t="n"/>
       <c r="K18" s="20" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="22" t="inlineStr">
-        <is>
-          <t>CBAM</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Netýká se (kapitola 40). ⚠ ADITEG s.r.o. však v registru CBAM chybí – viz poznámky.</t>
-        </is>
-      </c>
-      <c r="G19" s="20" t="n"/>
-      <c r="H19" s="21" t="n"/>
-      <c r="I19" s="20" t="n"/>
-      <c r="J19" s="20" t="n"/>
-      <c r="K19" s="20" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1211,7 +1155,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>HS kód (CCT/VPV KN)</t>
+          <t>HS kód</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -1523,7 +1467,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>4016910000</t>
+          <t>4008219000</t>
         </is>
       </c>
       <c r="G7" s="4" t="n">
@@ -1573,7 +1517,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>4016910000</t>
+          <t>4008219000</t>
         </is>
       </c>
       <c r="G8" s="4" t="n">
@@ -1973,7 +1917,7 @@
       </c>
       <c r="F16" s="14" t="inlineStr">
         <is>
-          <t>4016910000</t>
+          <t>4008219000</t>
         </is>
       </c>
       <c r="G16" s="15" t="n">
@@ -2034,7 +1978,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A109"/>
+  <dimension ref="A1:A96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -2318,30 +2262,30 @@
       <c r="A43" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="30" t="inlineStr">
-        <is>
-          <t>⚠ SAZEBNÍ ZAŘAZENÍ – POUŽITO PRAVIDLO CCT/VPV KN</t>
+      <c r="A44" s="27" t="inlineStr">
+        <is>
+          <t>SAZEBNÍ ZAŘAZENÍ – JEDEN HS KÓD PRO CELOU ZÁSILKU: 4008 21 90</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>V podkladech (faktury, packing listy, B/L) NENÍ uveden žádný HS kód – B/L popisuje zboží jen jako</t>
+          <t>Celá zásilka (všechny tři JSD, všech 15 fakturačních položek) je zařazena pod jediný kód</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>„RUBBER SHEET“. Oba níže uvedené kódy jsem odvodila pravidlem CCT/VPV KN podle</t>
+          <t>4008 21 90 – zadáno deklarantem. HS kód není v podkladech odesílatele nikde uveden</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>reference/Common_Customs_Tariff_EU_CZ.pptx. Takto zařazené položky:</t>
+          <t>(faktury, packing listy ani B/L jej neobsahují; B/L popisuje zboží jen jako „RUBBER SHEET“).</t>
         </is>
       </c>
     </row>
@@ -2351,393 +2295,302 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>A) 4008 21 90 – art. 0231268, 0230179, 0231419, 0230264, 0234614, 0230540, 0232061,</t>
+          <t>Znění kódu: TŘÍDA VII – kapitola 40 „Kaučuk a výrobky z něj“, číslo 4008 „Desky, listy, pásy, tyče</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">   0232184, 0231843, 0231842, 0230301</t>
+          <t>a profily z vulkanizovaného kaučuku, jiného než tvrdého kaučuku“, podpoložka 4008 21 (z nelehčeného</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">   CO TO JE? Desky / pásy z vulkanizovaného kaučuku v rolích, černé, 65 ±5 ShA, 2-3 a 7-8 MPa, tl. 3–20 mm.</t>
+          <t>kaučuku – desky, listy a pásy), KN 4008 21 90 (ostatní).</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Z ČEHO TO JE? Vulkanizovaný nelehčený kaučuk SBR / EPDM; u tří položek 1 textilní vložka (fabric) jako výztuž.</t>
-        </is>
-      </c>
+      <c r="A52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">   K ČEMU SLOUŽÍ? Technická pryž – těsnění, obklady, podložky; polotovar dodávaný v rolích k dalšímu zpracování.</t>
+          <t>Odpovídá zboží v zásilce: desky a pásy z vulkanizovaného nelehčeného kaučuku SBR / EPDM v rolích,</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Postup: TŘÍDA VII (plasty, kaučuk a pryž) → kapitola 40 → úvodní poznámky ke kap. 40 zboží nevylučují →</t>
+          <t>černé, 65 ±5 ShA, 2-3 a 7-8 MPa, tloušťka 3–20 mm, u části položek s 1 textilní vložkou (fabric)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">   číslo 4008 „Desky, listy, pásy, tyče a profily z vulkanizovaného kaučuku, jiného než tvrdého kaučuku“ →</t>
+          <t>jako výztuží – ta podle VPV 3(b) nemění podstatný charakter, ten dává kaučuk.</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   podpoložka 4008 21 (z nelehčeného kaučuku – desky, listy a pásy) → KN 4008 21 90 (ostatní). VPV 1 a VPV 6.</t>
-        </is>
-      </c>
+      <c r="A56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Textilní vložka: podle VPV 3(b) dává podstatný charakter kaučuk (výrazně převažuje hmotnostně, vložka</t>
+          <t>Pro pořádek k dohledání: u kamínkových desek (art. 0230559, 0230564) a rýhované desky (art. 0230238)</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">   plní pouze vyztužovací funkci) → zůstává v kap. 40, nikoli v kap. 59.</t>
+          <t>přicházelo v úvahu také číslo 4016 91 00 „Podlahové krytiny a rohože“. Deklarant rozhodl, že celá</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr"/>
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>zásilka jde pod 4008 21 90 – jednotné zařazení odpovídá tomu, že zboží je dodáváno v rolích jako</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>B) 4016 91 00 – art. 0230559, 0230564, 0230238</t>
+          <t>materiál, nikoli jako hotová rohož. Uvedeno pouze jako záznam o zvážené alternativě.</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   CO TO JE? Podlahové rohože z pryže – kamínková deska, kamínková deska speciál, rýhovaná deska.</t>
-        </is>
-      </c>
+      <c r="A61" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Z ČEHO TO JE? Vulkanizovaný nelehčený kaučuk (pryž).</t>
+      <c r="A62" s="28" t="inlineStr">
+        <is>
+          <t>⚠ PREFERENČNÍ PŮVOD A REX – OBOJÍ CHYBÍ</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">   K ČEMU SLOUŽÍ? Podlahová krytina / rohož – stájové a protiskluzové podlahy (Horse Rubber mat, Stable Mat).</t>
+          <t>PREFERENČNÍ VĚTA: NENÍ uvedena v žádném z dokladů. Zkontrolovány obě faktury, oba packing listy i B/L.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Postup: TŘÍDA VII → kapitola 40 → číslo 4016 „Ostatní výrobky z vulkanizovaného kaučuku, jiného než</t>
+          <t>REX ČÍSLO: NENÍ na žádné z faktur uvedeno. Faktury neobsahují číslo registrovaného vývozce</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">   tvrdého kaučuku“ → KN 4016 91 00 „Podlahové krytiny a rohože“. Podle VPV 3(a) má konkrétnější popis</t>
+          <t>ani jiné číslo celního povolení vývozce.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">   (hotová podlahová krytina) přednost před obecným číslem 4008 pro desky a pásy.</t>
+          <t>Země původu: Čína (CN). EU nemá s ČLR dohodu o preferenčním obchodu, preferenční sazba proto</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr"/>
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>není možná ani při doložení prohlášení – uplatní se standardní třetizemní clo (erga omnes).</t>
+        </is>
+      </c>
     </row>
     <row r="68">
-      <c r="A68" s="30" t="inlineStr">
-        <is>
-          <t>⚠ NEJISTOTA – DOPORUČUJI KONZULTOVAT</t>
+      <c r="A68" s="29" t="inlineStr">
+        <is>
+          <t>→ Sazbu k oběma HS kódům ověřit v TARIC k datu propuštění zboží.</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>1) Hranice 4008 vs. 4016 u art. 0230559 (3 mm Kamínková deska, dodávaná v roli 1,2 × 10 m) – rozměr</t>
-        </is>
-      </c>
+      <c r="A69" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   odpovídá spíše roli materiálu než hotové rohoži. Zařazeno do 4016 91 00 podle účelu (stájová rohož).</t>
+      <c r="A70" s="30" t="inlineStr">
+        <is>
+          <t>CBAM</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2) Položky s textilní vložkou – hranice kap. 40 vs. 5906. Zařazeno do 4008 21 90.</t>
+          <t>Zásilka NEOBSAHUJE žádnou CBAM položku – kaučuk a pryž (kapitola 40) nejsou v příloze I nařízení CBAM</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="29" t="inlineStr">
-        <is>
-          <t>→ Před podáním doporučuji potvrdit v TARIC, případně konzultovat tarifní tým: customs.tariff@mauriceward.com</t>
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>(CBAM = cement, elektřina, hnojiva, železo a ocel, hliník, vodík). Kód Y128/Y238/Y137 se na žádné JSD neuvádí.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">   (tento krok jsem zatím neprovedla – rozhodni prosím Ty).</t>
+          <t>Pro pořádek prověřeno v reference/CBAM_receivers_CZ.xlsx (list List1):</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr"/>
+      <c r="A74" s="31" t="inlineStr">
+        <is>
+          <t>⚠ ADITEG s.r.o. (EORI CZ26905710) V REGISTRU NENÍ – ani podle názvu firmy, ani podle EORI.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
-      <c r="A75" s="28" t="inlineStr">
-        <is>
-          <t>⚠ PREFERENČNÍ PŮVOD A REX – OBOJÍ CHYBÍ</t>
+      <c r="A75" s="29" t="inlineStr">
+        <is>
+          <t>→ Pro tuto zásilku to nevadí (žádné CBAM zboží). Pokud by ADITEG někdy dovážel CBAM zboží, je nutné</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>PREFERENČNÍ VĚTA: NENÍ uvedena v žádném z dokladů. Zkontrolovány obě faktury, oba packing listy i B/L.</t>
+          <t xml:space="preserve">   nejdřív zjistit jeho CBAM status a doplnit ho do registru. Status nedomýšlet.</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>REX ČÍSLO: NENÍ na žádné z faktur uvedeno. Faktury neobsahují číslo registrovaného vývozce</t>
-        </is>
-      </c>
+      <c r="A77" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>ani jiné číslo celního povolení vývozce.</t>
+      <c r="A78" s="30" t="inlineStr">
+        <is>
+          <t>ANTIDUMPING</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Země původu: Čína (CN). EU nemá s ČLR dohodu o preferenčním obchodu, preferenční sazba proto</t>
+          <t>Pro desky a pásy z vulkanizovaného kaučuku (4008 21 90) původem z ČLR nebylo zjištěno žádné</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>není možná ani při doložení prohlášení – uplatní se standardní třetizemní clo (erga omnes).</t>
+          <t>platné antidumpingové ani vyrovnávací opatření. Ověřit v TARIC k datu podání JSD.</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="29" t="inlineStr">
-        <is>
-          <t>→ Sazbu k oběma HS kódům ověřit v TARIC k datu propuštění zboží.</t>
-        </is>
-      </c>
+      <c r="A81" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr"/>
+      <c r="A82" s="30" t="inlineStr">
+        <is>
+          <t>INCOTERM</t>
+        </is>
+      </c>
     </row>
     <row r="83">
-      <c r="A83" s="30" t="inlineStr">
-        <is>
-          <t>CBAM</t>
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>FOB Xingang (Tianjin), Čína – dle obou faktur. Na B/L „FREIGHT COLLECT“, což je s FOB v souladu.</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>Zásilka NEOBSAHUJE žádnou CBAM položku – kaučuk a pryž (kapitola 40) nejsou v příloze I nařízení CBAM</t>
+      <c r="A84" s="29" t="inlineStr">
+        <is>
+          <t>→ Do celní hodnoty je nutno připočíst náklady na přepravu a pojištění do místa vstupu do EU.</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>(CBAM = cement, elektřina, hnojiva, železo a ocel, hliník, vodík). Kód Y128/Y238/Y137 se na žádné JSD neuvádí.</t>
-        </is>
-      </c>
+      <c r="A85" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>Pro pořádek prověřeno v reference/CBAM_receivers_CZ.xlsx (list List1):</t>
+      <c r="A86" s="28" t="inlineStr">
+        <is>
+          <t>⚠ NESROVNALOST V PODKLADECH – art. 0230564</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="31" t="inlineStr">
-        <is>
-          <t>⚠ ADITEG s.r.o. (EORI CZ26905710) V REGISTRU NENÍ – ani podle názvu firmy, ani podle EORI.</t>
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Faktura uvádí „17 mm Kamínková deska spec.“, packing list v popisu „12 mm Kamínková deska spec.“,</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="29" t="inlineStr">
-        <is>
-          <t>→ Pro tuto zásilku to nevadí (žádné CBAM zboží). Pokud by ADITEG někdy dovážel CBAM zboží, je nutné</t>
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>přičemž rozměr je v obou dokladech 1,22 x 1,83 m x 17 mm. V tabulce je použit popis z faktury (17 mm).</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   nejdřív zjistit jeho CBAM status a doplnit ho do registru. Status nedomýšlet.</t>
+      <c r="A89" s="29" t="inlineStr">
+        <is>
+          <t>→ Vyjasnit s odesílatelem před podáním – údaj jde do popisu zboží v kolonce 31.</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr"/>
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Kontrola množství: 446,52 m² / (1,22 × 1,83 m) = přesně 200 ks – souhlasí s packing listem.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
-      <c r="A91" s="30" t="inlineStr">
-        <is>
-          <t>ANTIDUMPING</t>
-        </is>
-      </c>
+      <c r="A91" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>Pro desky a rohože z vulkanizovaného kaučuku (4008 21, 4016 91) původem z ČLR nebylo zjištěno</t>
+      <c r="A92" s="27" t="inlineStr">
+        <is>
+          <t>POZNÁMKA K POPISU ZBOŽÍ A KE SLUČOVÁNÍ</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>žádné platné antidumpingové ani vyrovnávací opatření. Ověřit v TARIC k datu podání JSD.</t>
+          <t>Popisy v tabulce jsou převzaty doslovně z faktur (česky), bez úprav a bez přeformulování.</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr"/>
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Celá zásilka má jeden HS kód 4008 21 90, na každé JSD proto vychází jediný řádek. Stejný kód je na JSD 1</t>
+        </is>
+      </c>
     </row>
     <row r="95">
-      <c r="A95" s="30" t="inlineStr">
-        <is>
-          <t>INCOTERM</t>
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>i na JSD 2 samostatně – jde o dvě různá celní prohlášení, nelze je slučovat napříč JSD.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
-        <is>
-          <t>FOB Xingang (Tianjin), Čína – dle obou faktur. Na B/L „FREIGHT COLLECT“, což je s FOB v souladu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="29" t="inlineStr">
-        <is>
-          <t>→ Do celní hodnoty je nutno připočíst náklady na přepravu a pojištění do místa vstupu do EU.</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="inlineStr"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="28" t="inlineStr">
-        <is>
-          <t>⚠ NESROVNALOST V PODKLADECH – art. 0230564</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>Faktura uvádí „17 mm Kamínková deska spec.“, packing list v popisu „12 mm Kamínková deska spec.“,</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
-        <is>
-          <t>přičemž rozměr je v obou dokladech 1,22 x 1,83 m x 17 mm. V tabulce je použit popis z faktury (17 mm).</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="29" t="inlineStr">
-        <is>
-          <t>→ Vyjasnit s odesílatelem před podáním – údaj jde do popisu zboží v kolonce 31.</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>Kontrola množství: 446,52 m² / (1,22 × 1,83 m) = přesně 200 ks – souhlasí s packing listem.</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="27" t="inlineStr">
-        <is>
-          <t>POZNÁMKA K POPISU ZBOŽÍ A KE SLUČOVÁNÍ</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>Popisy v tabulce jsou převzaty doslovně z faktur (česky), bez úprav a bez přeformulování.</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>Položky jsou sloučeny na unikátní HS kódy v rámci každého JSD. Stejný HS kód 4008 21 90 je na JSD 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>i na JSD 2 samostatně – jde o dvě různá celní prohlášení, nelze je slučovat napříč JSD.</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
         <is>
           <t>Odesílatel je u celé zásilky jeden (Qingdao Conet), dělení podle odesílatele proto nebylo potřeba.</t>
         </is>

</xml_diff>

<commit_message>
Shorten goods descriptions on the HS Summary sheet
Keep material (SBR / EPDM), form (sheet, sheet with textile ply,
stud / ribbed mat) and dimensions; drop hardness (65 +/- 5 Sh) and
tensile strength (2-3 / 7-8 MPa), which do not affect classification
under 4008 21 90.

The verbatim Czech invoice descriptions stay unchanged on the
"Polozky (detail)" sheet so the wording can still be matched against
the invoice during a check.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EgFygQDzpiBueVLaTVai9C
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_ADITEG_CZ26009365.xlsx
+++ b/output/HS_Code_Summary_ADITEG_CZ26009365.xlsx
@@ -596,7 +596,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Popis zboží (CZ) – doslovně z faktury</t>
+          <t>Popis zboží (CZ) – zkrácený</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -663,13 +663,13 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>0231268 – EPDM/SBR 65 +/- 5 Sh., černá, 2-3 MPa 3 mm, 2 x 10 m
-0230179 – SBR 65 +/- 5 Sh.černá, 2-3 MPa 5 mm x 1.200 x 10.000 mm
-0231419 – SBR 65 +/- 5 Sh.černá, 2-3 MPa 6 mm x 2.000 x 10.000 mm
-0230264 – SBR 65 +/- 5 Sh.černá, 2-3 MPa, 1 vložka(fabric) 10 mm x 1.200 x 10.000 mm
-0234614 – SBR 65 +/-5SHA  černá, 2-3 MPa 8 mm x1.600 x 10.000 mm
-0230559 – 3 mm Kamínková deska.(Horse Rubber mat) 3 mm x 1.200 x 10.000 mm
-0230564 – 17 mm Kamínková deska spec.（Round button Stable Mat）Kamínková deska - speciál 1,22 x 1,83 m x 17 mm</t>
+          <t>0231268 – EPDM/SBR deska 3 mm, 2 x 10 m
+0230179 – SBR deska 5 mm x 1.200 x 10.000 mm
+0231419 – SBR deska 6 mm x 2.000 x 10.000 mm
+0230264 – SBR deska s 1 textilní vložkou 10 mm x 1.200 x 10.000 mm
+0234614 – SBR deska 8 mm x 1.600 x 10.000 mm
+0230559 – Kamínková deska 3 mm x 1.200 x 10.000 mm
+0230564 – Kamínková deska speciál 1,22 x 1,83 m x 17 mm</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -755,13 +755,13 @@
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>0230540 – EPDM/SBR 65 +/- 5 Sh.černá, 7-8 MPa 5mm x 1.200 x 10.000 mm
-0232061 – SBR 65 +/- 5 Sh. černá, 2-3 MPa 20 mm x 1.400 x 10.000 mm
-0232184 – SBR 65+/-5SHAčerná, 2-3 MPa, 1 vložky(fabirc)3mm x 1.400 x 10.000 mm
-0231843 – SBR  65+/5SHA černá, 2-3 MPa, 10mm x 1.200 x 25.000 mm
-0231842 – SBR 65 +/- 5 Sh.černá, 2-3 MPa 10 mm x 1.200 x 13.000 mm
-0230264 – SBR 65 +/- 5 Sh. černá, 2-3 MPa, 1 vložka(fabric) 10 mm x 1.200 x 10.000 mm
-0230301 – EPDM/SBR 65 +/- 5 ShA černá, 2-3 MPa, 1 vložka 8 mm x 1.200 x 10.000 mm</t>
+          <t>0230540 – EPDM/SBR deska 5 mm x 1.200 x 10.000 mm
+0232061 – SBR deska 20 mm x 1.400 x 10.000 mm
+0232184 – SBR deska s 1 textilní vložkou 3 mm x 1.400 x 10.000 mm
+0231843 – SBR deska 10 mm x 1.200 x 25.000 mm
+0231842 – SBR deska 10 mm x 1.200 x 13.000 mm
+0230264 – SBR deska s 1 textilní vložkou 10 mm x 1.200 x 10.000 mm
+0230301 – EPDM/SBR deska s 1 textilní vložkou 8 mm x 1.200 x 10.000 mm</t>
         </is>
       </c>
       <c r="F4" s="10" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="E6" s="13" t="inlineStr">
         <is>
-          <t>0230238 – Fine ribbed mat(Rýhovaná deska - malá) 3mm，1.2X10m</t>
+          <t>0230238 – Rýhovaná deska 3 mm, 1,2 x 10 m</t>
         </is>
       </c>
       <c r="F6" s="14" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Doslovný český popis z faktury, bez úprav.</t>
+          <t>Zde zkrácený popis (materiál, provedení, rozměr). Doslovný popis z faktury je na listu „Položky (detail)“.</t>
         </is>
       </c>
       <c r="G17" s="20" t="n"/>
@@ -1978,7 +1978,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A96"/>
+  <dimension ref="A1:A100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -2571,26 +2571,54 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Popisy v tabulce jsou převzaty doslovně z faktur (česky), bez úprav a bez přeformulování.</t>
+          <t>Popisy na listu „HS Summary“ jsou zkrácené – ponechán materiál (SBR / EPDM), provedení (deska, deska</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Celá zásilka má jeden HS kód 4008 21 90, na každé JSD proto vychází jediný řádek. Stejný kód je na JSD 1</t>
+          <t>s textilní vložkou, kamínková / rýhovaná deska) a rozměr. Vypuštěna tvrdost (65 ±5 Sh) a pevnost</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>i na JSD 2 samostatně – jde o dvě různá celní prohlášení, nelze je slučovat napříč JSD.</t>
+          <t>(2-3 / 7-8 MPa), které nejsou pro zařazení do 4008 21 90 rozhodující.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
+        <is>
+          <t>Doslovné české popisy z faktur zůstávají beze změny na listu „Položky (detail)“ – pro doložení</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>shody s fakturou při kontrole.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Celá zásilka má jeden HS kód 4008 21 90, na každé JSD proto vychází jediný řádek. Stejný kód je na JSD 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>i na JSD 2 samostatně – jde o dvě různá celní prohlášení, nelze je slučovat napříč JSD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
         <is>
           <t>Odesílatel je u celé zásilky jeden (Qingdao Conet), dělení podle odesílatele proto nebylo potřeba.</t>
         </is>

</xml_diff>